<commit_message>
Added multi-processing for mesh_template_track_node.py Fixed zooming problem before panning in bandpass_filter_node.py Fixed project-saving-loading-time-too-long problem (by caching related-absolute path result) Fixed bugs in image_sequence_node about edited file list (for load/save project).
</commit_message>
<xml_diff>
--- a/samples/signals/signals02.xlsx
+++ b/samples/signals/signals02.xlsx
@@ -450,7 +450,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1791258022.4191296</t>
+          <t>1791279039.124181</t>
         </is>
       </c>
     </row>
@@ -462,7 +462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -588,7 +588,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>{"common": {"duration": 5.0, "dt": 0.01}, "sine_channels": [{"enabled": true, "amplitude": 1.0, "frequency": 1.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": true, "amplitude": 2.0, "frequency": 2.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 5.0, "frequency": 20.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 5.0, "frequency": 15.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 5.0, "frequency": 12.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 5.0, "frequency": 25.0, "decay": 0.0, "time_shift": 0.0}], "noise_channel": {"enabled": false, "distribution": "gaussian", "amplitude": 5.0, "seed": 0}}</t>
+          <t>{"common": {"duration": 5.0, "dt": 0.01}, "sine_channels": [{"enabled": true, "amplitude": 1.0, "frequency": 1.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": true, "amplitude": 2.0, "frequency": 2.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 5.0, "frequency": 20.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 5.0, "frequency": 15.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 5.0, "frequency": 12.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 5.0, "frequency": 25.0, "decay": 0.0, "time_shift": 0.0}], "noise_channel": {"enabled": true, "distribution": "gaussian", "amplitude": 0.2, "seed": 0}}</t>
         </is>
       </c>
     </row>
@@ -609,10 +609,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>348</v>
+        <v>872</v>
       </c>
       <c r="E3" t="n">
-        <v>320</v>
+        <v>101</v>
       </c>
       <c r="F3" t="n">
         <v>160</v>
@@ -697,204 +697,34 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>node_5</t>
+          <t>node_8</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>array_input</t>
+          <t>cwt_1d</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Array Input</t>
+          <t>CWT (1D)</t>
         </is>
       </c>
       <c r="D6" t="n">
+        <v>475</v>
+      </c>
+      <c r="E6" t="n">
         <v>536</v>
       </c>
-      <c r="E6" t="n">
-        <v>39</v>
-      </c>
       <c r="F6" t="n">
-        <v>220</v>
+        <v>150</v>
       </c>
       <c r="G6" t="n">
-        <v>220</v>
+        <v>130</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>{"csv": "115.75972\n114.39833\n97.27000\n107.99972\n104.57222\n\n\n\n", "dtype": "float64", "shape_mode": "manual", "shape_text": "-1"}</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>node_6</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>bandpass_filter</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Band-Pass Filter</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>894</v>
-      </c>
-      <c r="E7" t="n">
-        <v>204</v>
-      </c>
-      <c r="F7" t="n">
-        <v>160</v>
-      </c>
-      <c r="G7" t="n">
-        <v>110</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>{"filter": {"mode": "bandpass", "f_low": 0.5, "f_high": 5.0, "order": 4.0, "shape": "butterworth", "remove_mean": true, "pad_frac": 0.1}, "signal_index": 0, "show_db": false}</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>node_8</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>cwt_1d</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CWT (1D)</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>475</v>
-      </c>
-      <c r="E8" t="n">
-        <v>536</v>
-      </c>
-      <c r="F8" t="n">
-        <v>150</v>
-      </c>
-      <c r="G8" t="n">
-        <v>130</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
           <t>{"wavelet_family": "morl", "wavelet_params": {"bandwidth": 1.5, "center_freq": 1.0, "order": 2}, "scale_settings": {"scale_min": 1.0, "scale_max": 64.0, "num_scales": 40, "spacing": "log"}, "view_mode": "magnitude", "y_axis_mode": "frequency", "log_color": false, "y_log_scale": true, "colormap": "viridis"}</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>node_9</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>signal_generator</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Signal Generator</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>367</v>
-      </c>
-      <c r="E9" t="n">
-        <v>84</v>
-      </c>
-      <c r="F9" t="n">
-        <v>150</v>
-      </c>
-      <c r="G9" t="n">
-        <v>110</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>{"common": {"duration": 10.0, "dt": 0.01}, "sine_channels": [{"enabled": true, "amplitude": 1.0, "frequency": 1.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 1.0, "frequency": 2.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 1.0, "frequency": 3.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 1.0, "frequency": 4.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 1.0, "frequency": 5.0, "decay": 0.0, "time_shift": 0.0}, {"enabled": false, "amplitude": 1.0, "frequency": 6.0, "decay": 0.0, "time_shift": 0.0}], "noise_channel": {"enabled": false, "distribution": "gaussian", "amplitude": 0.05, "seed": 0}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>node_10</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>time_sync</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Time Sync</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>47</v>
-      </c>
-      <c r="E10" t="n">
-        <v>217</v>
-      </c>
-      <c r="F10" t="n">
-        <v>150</v>
-      </c>
-      <c r="G10" t="n">
-        <v>130</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>{"t_shift_applied": 0.0, "slider_min": -1.0, "slider_max": 1.0, "interp_method": "linear", "diff_order": 0, "error_metric": "rmse", "normalize_error": true, "show_normalized_plot": false, "style": {"series1": {"color": "#1f77b4", "line_width": 1.5, "marker": "None", "marker_size": 4, "marker_color": "#1f77b4"}, "series2": {"color": "#d62728", "line_width": 1.5, "marker": "None", "marker_size": 4, "marker_color": "#d62728"}, "legend_on": true}}</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>node_11</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>stereo_sync</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Stereo Sync</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>920</v>
-      </c>
-      <c r="E11" t="n">
-        <v>452</v>
-      </c>
-      <c r="F11" t="n">
-        <v>160</v>
-      </c>
-      <c r="G11" t="n">
-        <v>270</v>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>{"t_shift_applied": [], "slider_min": -1.0, "slider_max": 1.0, "nan_fill_method": "none (exclude gaps)", "interp_method": "linear", "excluded_points": [], "aggregation": "median", "outlier_threshold": null}</t>
         </is>
       </c>
     </row>

</xml_diff>